<commit_message>
feat(ai): purge grand and expensive from master gold emotion codebook
</commit_message>
<xml_diff>
--- a/data/analyze/nrc8_words_included.xlsx
+++ b/data/analyze/nrc8_words_included.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2298" uniqueCount="734">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2278" uniqueCount="733">
   <si>
     <t>word</t>
   </si>
@@ -2051,9 +2051,6 @@
   </si>
   <si>
     <t>positive</t>
-  </si>
-  <si>
-    <t>None</t>
   </si>
   <si>
     <t>negative, positive</t>
@@ -2637,7 +2634,7 @@
         <v>678</v>
       </c>
       <c r="J2" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -2669,7 +2666,7 @@
         <v>678</v>
       </c>
       <c r="J3" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -2701,7 +2698,7 @@
         <v>678</v>
       </c>
       <c r="J4" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -2733,7 +2730,7 @@
         <v>678</v>
       </c>
       <c r="J5" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -2765,7 +2762,7 @@
         <v>678</v>
       </c>
       <c r="J6" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -2797,7 +2794,7 @@
         <v>678</v>
       </c>
       <c r="J7" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -2825,9 +2822,6 @@
       <c r="H8" t="s">
         <v>638</v>
       </c>
-      <c r="I8" t="s">
-        <v>679</v>
-      </c>
       <c r="J8" t="s">
         <v>638</v>
       </c>
@@ -2861,7 +2855,7 @@
         <v>678</v>
       </c>
       <c r="J9" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -2893,7 +2887,7 @@
         <v>678</v>
       </c>
       <c r="J10" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -2925,7 +2919,7 @@
         <v>678</v>
       </c>
       <c r="J11" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -2957,7 +2951,7 @@
         <v>678</v>
       </c>
       <c r="J12" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -2989,7 +2983,7 @@
         <v>678</v>
       </c>
       <c r="J13" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -3021,7 +3015,7 @@
         <v>678</v>
       </c>
       <c r="J14" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -3053,7 +3047,7 @@
         <v>678</v>
       </c>
       <c r="J15" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -3085,7 +3079,7 @@
         <v>678</v>
       </c>
       <c r="J16" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -3117,7 +3111,7 @@
         <v>89</v>
       </c>
       <c r="J17" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -3149,7 +3143,7 @@
         <v>89</v>
       </c>
       <c r="J18" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -3178,10 +3172,10 @@
         <v>84</v>
       </c>
       <c r="I19" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="J19" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -3213,7 +3207,7 @@
         <v>678</v>
       </c>
       <c r="J20" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -3245,7 +3239,7 @@
         <v>678</v>
       </c>
       <c r="J21" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -3277,7 +3271,7 @@
         <v>678</v>
       </c>
       <c r="J22" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -3309,7 +3303,7 @@
         <v>89</v>
       </c>
       <c r="J23" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -3341,7 +3335,7 @@
         <v>678</v>
       </c>
       <c r="J24" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -3373,7 +3367,7 @@
         <v>678</v>
       </c>
       <c r="J25" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -3405,7 +3399,7 @@
         <v>89</v>
       </c>
       <c r="J26" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -3437,7 +3431,7 @@
         <v>678</v>
       </c>
       <c r="J27" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -3469,7 +3463,7 @@
         <v>89</v>
       </c>
       <c r="J28" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -3501,7 +3495,7 @@
         <v>678</v>
       </c>
       <c r="J29" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -3529,9 +3523,6 @@
       <c r="H30" t="s">
         <v>644</v>
       </c>
-      <c r="I30" t="s">
-        <v>679</v>
-      </c>
       <c r="J30" t="s">
         <v>644</v>
       </c>
@@ -3565,7 +3556,7 @@
         <v>678</v>
       </c>
       <c r="J31" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -3597,7 +3588,7 @@
         <v>678</v>
       </c>
       <c r="J32" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -3625,9 +3616,6 @@
       <c r="H33" t="s">
         <v>42</v>
       </c>
-      <c r="I33" t="s">
-        <v>679</v>
-      </c>
       <c r="J33" t="s">
         <v>42</v>
       </c>
@@ -3661,7 +3649,7 @@
         <v>678</v>
       </c>
       <c r="J34" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="35" spans="1:10">
@@ -3693,7 +3681,7 @@
         <v>678</v>
       </c>
       <c r="J35" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -3721,9 +3709,6 @@
       <c r="H36" t="s">
         <v>649</v>
       </c>
-      <c r="I36" t="s">
-        <v>679</v>
-      </c>
       <c r="J36" t="s">
         <v>649</v>
       </c>
@@ -3757,7 +3742,7 @@
         <v>678</v>
       </c>
       <c r="J37" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -3789,7 +3774,7 @@
         <v>678</v>
       </c>
       <c r="J38" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -3821,7 +3806,7 @@
         <v>678</v>
       </c>
       <c r="J39" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="40" spans="1:10">
@@ -3853,7 +3838,7 @@
         <v>678</v>
       </c>
       <c r="J40" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="41" spans="1:10">
@@ -3885,7 +3870,7 @@
         <v>678</v>
       </c>
       <c r="J41" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="42" spans="1:10">
@@ -3913,9 +3898,6 @@
       <c r="H42" t="s">
         <v>651</v>
       </c>
-      <c r="I42" t="s">
-        <v>679</v>
-      </c>
       <c r="J42" t="s">
         <v>651</v>
       </c>
@@ -3949,7 +3931,7 @@
         <v>678</v>
       </c>
       <c r="J43" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="44" spans="1:10">
@@ -3981,7 +3963,7 @@
         <v>678</v>
       </c>
       <c r="J44" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="45" spans="1:10">
@@ -4013,7 +3995,7 @@
         <v>89</v>
       </c>
       <c r="J45" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="46" spans="1:10">
@@ -4045,7 +4027,7 @@
         <v>89</v>
       </c>
       <c r="J46" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="47" spans="1:10">
@@ -4077,7 +4059,7 @@
         <v>678</v>
       </c>
       <c r="J47" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="48" spans="1:10">
@@ -4109,7 +4091,7 @@
         <v>678</v>
       </c>
       <c r="J48" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -4141,7 +4123,7 @@
         <v>678</v>
       </c>
       <c r="J49" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -4173,7 +4155,7 @@
         <v>678</v>
       </c>
       <c r="J50" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -4205,7 +4187,7 @@
         <v>678</v>
       </c>
       <c r="J51" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="52" spans="1:10">
@@ -4237,7 +4219,7 @@
         <v>678</v>
       </c>
       <c r="J52" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="53" spans="1:10">
@@ -4269,7 +4251,7 @@
         <v>89</v>
       </c>
       <c r="J53" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="54" spans="1:10">
@@ -4301,7 +4283,7 @@
         <v>89</v>
       </c>
       <c r="J54" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="55" spans="1:10">
@@ -4333,7 +4315,7 @@
         <v>89</v>
       </c>
       <c r="J55" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="56" spans="1:10">
@@ -4365,7 +4347,7 @@
         <v>678</v>
       </c>
       <c r="J56" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
     </row>
     <row r="57" spans="1:10">
@@ -4393,9 +4375,6 @@
       <c r="H57" t="s">
         <v>62</v>
       </c>
-      <c r="I57" t="s">
-        <v>679</v>
-      </c>
       <c r="J57" t="s">
         <v>62</v>
       </c>
@@ -4429,7 +4408,7 @@
         <v>678</v>
       </c>
       <c r="J58" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="59" spans="1:10">
@@ -4461,7 +4440,7 @@
         <v>678</v>
       </c>
       <c r="J59" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="60" spans="1:10">
@@ -4493,7 +4472,7 @@
         <v>89</v>
       </c>
       <c r="J60" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="61" spans="1:10">
@@ -4525,7 +4504,7 @@
         <v>678</v>
       </c>
       <c r="J61" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="62" spans="1:10">
@@ -4557,7 +4536,7 @@
         <v>89</v>
       </c>
       <c r="J62" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="63" spans="1:10">
@@ -4589,7 +4568,7 @@
         <v>678</v>
       </c>
       <c r="J63" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
     <row r="64" spans="1:10">
@@ -4621,7 +4600,7 @@
         <v>678</v>
       </c>
       <c r="J64" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
     </row>
     <row r="65" spans="1:10">
@@ -4653,7 +4632,7 @@
         <v>678</v>
       </c>
       <c r="J65" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="66" spans="1:10">
@@ -4685,7 +4664,7 @@
         <v>678</v>
       </c>
       <c r="J66" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="67" spans="1:10">
@@ -4717,7 +4696,7 @@
         <v>678</v>
       </c>
       <c r="J67" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="68" spans="1:10">
@@ -4749,7 +4728,7 @@
         <v>678</v>
       </c>
       <c r="J68" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="69" spans="1:10">
@@ -4781,7 +4760,7 @@
         <v>678</v>
       </c>
       <c r="J69" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="70" spans="1:10">
@@ -4813,7 +4792,7 @@
         <v>678</v>
       </c>
       <c r="J70" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="71" spans="1:10">
@@ -4845,7 +4824,7 @@
         <v>89</v>
       </c>
       <c r="J71" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="72" spans="1:10">
@@ -4877,7 +4856,7 @@
         <v>678</v>
       </c>
       <c r="J72" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="73" spans="1:10">
@@ -4909,7 +4888,7 @@
         <v>678</v>
       </c>
       <c r="J73" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="74" spans="1:10">
@@ -4941,7 +4920,7 @@
         <v>678</v>
       </c>
       <c r="J74" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="75" spans="1:10">
@@ -4973,7 +4952,7 @@
         <v>678</v>
       </c>
       <c r="J75" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="76" spans="1:10">
@@ -5005,7 +4984,7 @@
         <v>678</v>
       </c>
       <c r="J76" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="77" spans="1:10">
@@ -5037,7 +5016,7 @@
         <v>678</v>
       </c>
       <c r="J77" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="78" spans="1:10">
@@ -5069,7 +5048,7 @@
         <v>678</v>
       </c>
       <c r="J78" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="79" spans="1:10">
@@ -5101,7 +5080,7 @@
         <v>89</v>
       </c>
       <c r="J79" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="80" spans="1:10">
@@ -5133,7 +5112,7 @@
         <v>89</v>
       </c>
       <c r="J80" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="81" spans="1:10">
@@ -5165,7 +5144,7 @@
         <v>89</v>
       </c>
       <c r="J81" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="82" spans="1:10">
@@ -5197,7 +5176,7 @@
         <v>678</v>
       </c>
       <c r="J82" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="83" spans="1:10">
@@ -5229,7 +5208,7 @@
         <v>678</v>
       </c>
       <c r="J83" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="84" spans="1:10">
@@ -5261,7 +5240,7 @@
         <v>89</v>
       </c>
       <c r="J84" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="85" spans="1:10">
@@ -5293,7 +5272,7 @@
         <v>678</v>
       </c>
       <c r="J85" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="86" spans="1:10">
@@ -5325,7 +5304,7 @@
         <v>678</v>
       </c>
       <c r="J86" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="87" spans="1:10">
@@ -5357,7 +5336,7 @@
         <v>678</v>
       </c>
       <c r="J87" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="88" spans="1:10">
@@ -5389,7 +5368,7 @@
         <v>678</v>
       </c>
       <c r="J88" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="89" spans="1:10">
@@ -5421,7 +5400,7 @@
         <v>678</v>
       </c>
       <c r="J89" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="90" spans="1:10">
@@ -5453,7 +5432,7 @@
         <v>89</v>
       </c>
       <c r="J90" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="91" spans="1:10">
@@ -5485,7 +5464,7 @@
         <v>678</v>
       </c>
       <c r="J91" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="92" spans="1:10">
@@ -5517,7 +5496,7 @@
         <v>678</v>
       </c>
       <c r="J92" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="93" spans="1:10">
@@ -5545,9 +5524,6 @@
       <c r="H93" t="s">
         <v>658</v>
       </c>
-      <c r="I93" t="s">
-        <v>679</v>
-      </c>
       <c r="J93" t="s">
         <v>658</v>
       </c>
@@ -5581,7 +5557,7 @@
         <v>89</v>
       </c>
       <c r="J94" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="95" spans="1:10">
@@ -5610,10 +5586,10 @@
         <v>652</v>
       </c>
       <c r="I95" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="J95" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="96" spans="1:10">
@@ -5645,7 +5621,7 @@
         <v>678</v>
       </c>
       <c r="J96" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="97" spans="1:10">
@@ -5677,7 +5653,7 @@
         <v>678</v>
       </c>
       <c r="J97" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="98" spans="1:10">
@@ -5709,7 +5685,7 @@
         <v>678</v>
       </c>
       <c r="J98" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
     <row r="99" spans="1:10">
@@ -5741,7 +5717,7 @@
         <v>89</v>
       </c>
       <c r="J99" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="100" spans="1:10">
@@ -5773,7 +5749,7 @@
         <v>678</v>
       </c>
       <c r="J100" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
     </row>
     <row r="101" spans="1:10">
@@ -5805,7 +5781,7 @@
         <v>89</v>
       </c>
       <c r="J101" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="102" spans="1:10">
@@ -5837,7 +5813,7 @@
         <v>678</v>
       </c>
       <c r="J102" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="103" spans="1:10">
@@ -5869,7 +5845,7 @@
         <v>678</v>
       </c>
       <c r="J103" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="104" spans="1:10">
@@ -5901,7 +5877,7 @@
         <v>89</v>
       </c>
       <c r="J104" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="105" spans="1:10">
@@ -5933,7 +5909,7 @@
         <v>678</v>
       </c>
       <c r="J105" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="106" spans="1:10">
@@ -5965,7 +5941,7 @@
         <v>89</v>
       </c>
       <c r="J106" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="107" spans="1:10">
@@ -5997,7 +5973,7 @@
         <v>678</v>
       </c>
       <c r="J107" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="108" spans="1:10">
@@ -6029,7 +6005,7 @@
         <v>678</v>
       </c>
       <c r="J108" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="109" spans="1:10">
@@ -6057,9 +6033,6 @@
       <c r="H109" t="s">
         <v>638</v>
       </c>
-      <c r="I109" t="s">
-        <v>679</v>
-      </c>
       <c r="J109" t="s">
         <v>638</v>
       </c>
@@ -6093,7 +6066,7 @@
         <v>89</v>
       </c>
       <c r="J110" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
     </row>
     <row r="111" spans="1:10">
@@ -6125,7 +6098,7 @@
         <v>678</v>
       </c>
       <c r="J111" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="112" spans="1:10">
@@ -6157,7 +6130,7 @@
         <v>678</v>
       </c>
       <c r="J112" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="113" spans="1:10">
@@ -6189,7 +6162,7 @@
         <v>89</v>
       </c>
       <c r="J113" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="114" spans="1:10">
@@ -6221,7 +6194,7 @@
         <v>89</v>
       </c>
       <c r="J114" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="115" spans="1:10">
@@ -6253,7 +6226,7 @@
         <v>678</v>
       </c>
       <c r="J115" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="116" spans="1:10">
@@ -6285,7 +6258,7 @@
         <v>89</v>
       </c>
       <c r="J116" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="117" spans="1:10">
@@ -6313,9 +6286,6 @@
       <c r="H117" t="s">
         <v>650</v>
       </c>
-      <c r="I117" t="s">
-        <v>679</v>
-      </c>
       <c r="J117" t="s">
         <v>650</v>
       </c>
@@ -6349,7 +6319,7 @@
         <v>678</v>
       </c>
       <c r="J118" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="119" spans="1:10">
@@ -6381,7 +6351,7 @@
         <v>89</v>
       </c>
       <c r="J119" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="120" spans="1:10">
@@ -6413,7 +6383,7 @@
         <v>678</v>
       </c>
       <c r="J120" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="121" spans="1:10">
@@ -6445,7 +6415,7 @@
         <v>678</v>
       </c>
       <c r="J121" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="122" spans="1:10">
@@ -6477,7 +6447,7 @@
         <v>678</v>
       </c>
       <c r="J122" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="123" spans="1:10">
@@ -6509,7 +6479,7 @@
         <v>89</v>
       </c>
       <c r="J123" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="124" spans="1:10">
@@ -6541,7 +6511,7 @@
         <v>89</v>
       </c>
       <c r="J124" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="125" spans="1:10">
@@ -6573,7 +6543,7 @@
         <v>89</v>
       </c>
       <c r="J125" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="126" spans="1:10">
@@ -6605,7 +6575,7 @@
         <v>89</v>
       </c>
       <c r="J126" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="127" spans="1:10">
@@ -6637,7 +6607,7 @@
         <v>89</v>
       </c>
       <c r="J127" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="128" spans="1:10">
@@ -6669,7 +6639,7 @@
         <v>678</v>
       </c>
       <c r="J128" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="129" spans="1:10">
@@ -6701,7 +6671,7 @@
         <v>678</v>
       </c>
       <c r="J129" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="130" spans="1:10">
@@ -6733,7 +6703,7 @@
         <v>89</v>
       </c>
       <c r="J130" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="131" spans="1:10">
@@ -6765,7 +6735,7 @@
         <v>678</v>
       </c>
       <c r="J131" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="132" spans="1:10">
@@ -6797,7 +6767,7 @@
         <v>89</v>
       </c>
       <c r="J132" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="133" spans="1:10">
@@ -6829,7 +6799,7 @@
         <v>678</v>
       </c>
       <c r="J133" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="134" spans="1:10">
@@ -6861,7 +6831,7 @@
         <v>89</v>
       </c>
       <c r="J134" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="135" spans="1:10">
@@ -6893,7 +6863,7 @@
         <v>89</v>
       </c>
       <c r="J135" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="136" spans="1:10">
@@ -6925,7 +6895,7 @@
         <v>678</v>
       </c>
       <c r="J136" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="137" spans="1:10">
@@ -6957,7 +6927,7 @@
         <v>678</v>
       </c>
       <c r="J137" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="138" spans="1:10">
@@ -6989,7 +6959,7 @@
         <v>678</v>
       </c>
       <c r="J138" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
     </row>
     <row r="139" spans="1:10">
@@ -7021,7 +6991,7 @@
         <v>678</v>
       </c>
       <c r="J139" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="140" spans="1:10">
@@ -7053,7 +7023,7 @@
         <v>678</v>
       </c>
       <c r="J140" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="141" spans="1:10">
@@ -7085,7 +7055,7 @@
         <v>678</v>
       </c>
       <c r="J141" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="142" spans="1:10">
@@ -7117,7 +7087,7 @@
         <v>89</v>
       </c>
       <c r="J142" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="143" spans="1:10">
@@ -7149,7 +7119,7 @@
         <v>678</v>
       </c>
       <c r="J143" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="144" spans="1:10">
@@ -7181,7 +7151,7 @@
         <v>678</v>
       </c>
       <c r="J144" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="145" spans="1:10">
@@ -7213,7 +7183,7 @@
         <v>678</v>
       </c>
       <c r="J145" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
     <row r="146" spans="1:10">
@@ -7241,9 +7211,6 @@
       <c r="H146" t="s">
         <v>650</v>
       </c>
-      <c r="I146" t="s">
-        <v>679</v>
-      </c>
       <c r="J146" t="s">
         <v>650</v>
       </c>
@@ -7277,7 +7244,7 @@
         <v>678</v>
       </c>
       <c r="J147" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="148" spans="1:10">
@@ -7309,7 +7276,7 @@
         <v>678</v>
       </c>
       <c r="J148" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="149" spans="1:10">
@@ -7341,7 +7308,7 @@
         <v>89</v>
       </c>
       <c r="J149" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="150" spans="1:10">
@@ -7373,7 +7340,7 @@
         <v>89</v>
       </c>
       <c r="J150" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="151" spans="1:10">
@@ -7405,7 +7372,7 @@
         <v>89</v>
       </c>
       <c r="J151" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="152" spans="1:10">
@@ -7433,9 +7400,6 @@
       <c r="H152" t="s">
         <v>42</v>
       </c>
-      <c r="I152" t="s">
-        <v>679</v>
-      </c>
       <c r="J152" t="s">
         <v>42</v>
       </c>
@@ -7469,7 +7433,7 @@
         <v>678</v>
       </c>
       <c r="J153" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="154" spans="1:10">
@@ -7501,7 +7465,7 @@
         <v>678</v>
       </c>
       <c r="J154" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="155" spans="1:10">
@@ -7529,9 +7493,6 @@
       <c r="H155" t="s">
         <v>42</v>
       </c>
-      <c r="I155" t="s">
-        <v>679</v>
-      </c>
       <c r="J155" t="s">
         <v>42</v>
       </c>
@@ -7565,7 +7526,7 @@
         <v>89</v>
       </c>
       <c r="J156" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="157" spans="1:10">
@@ -7597,7 +7558,7 @@
         <v>678</v>
       </c>
       <c r="J157" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="158" spans="1:10">
@@ -7629,7 +7590,7 @@
         <v>89</v>
       </c>
       <c r="J158" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="159" spans="1:10">
@@ -7661,7 +7622,7 @@
         <v>89</v>
       </c>
       <c r="J159" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="160" spans="1:10">
@@ -7693,7 +7654,7 @@
         <v>89</v>
       </c>
       <c r="J160" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="161" spans="1:10">
@@ -7725,7 +7686,7 @@
         <v>678</v>
       </c>
       <c r="J161" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
     </row>
     <row r="162" spans="1:10">
@@ -7757,7 +7718,7 @@
         <v>678</v>
       </c>
       <c r="J162" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="163" spans="1:10">
@@ -7789,7 +7750,7 @@
         <v>678</v>
       </c>
       <c r="J163" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="164" spans="1:10">
@@ -7821,7 +7782,7 @@
         <v>678</v>
       </c>
       <c r="J164" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="165" spans="1:10">
@@ -7853,7 +7814,7 @@
         <v>89</v>
       </c>
       <c r="J165" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="166" spans="1:10">
@@ -7885,7 +7846,7 @@
         <v>678</v>
       </c>
       <c r="J166" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="167" spans="1:10">
@@ -7917,7 +7878,7 @@
         <v>678</v>
       </c>
       <c r="J167" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="168" spans="1:10">
@@ -7949,7 +7910,7 @@
         <v>89</v>
       </c>
       <c r="J168" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="169" spans="1:10">
@@ -7981,7 +7942,7 @@
         <v>678</v>
       </c>
       <c r="J169" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="170" spans="1:10">
@@ -8013,7 +7974,7 @@
         <v>678</v>
       </c>
       <c r="J170" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="171" spans="1:10">
@@ -8045,7 +8006,7 @@
         <v>678</v>
       </c>
       <c r="J171" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="172" spans="1:10">
@@ -8077,7 +8038,7 @@
         <v>678</v>
       </c>
       <c r="J172" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="173" spans="1:10">
@@ -8109,7 +8070,7 @@
         <v>89</v>
       </c>
       <c r="J173" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="174" spans="1:10">
@@ -8141,7 +8102,7 @@
         <v>678</v>
       </c>
       <c r="J174" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="175" spans="1:10">
@@ -8173,7 +8134,7 @@
         <v>678</v>
       </c>
       <c r="J175" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="176" spans="1:10">
@@ -8205,7 +8166,7 @@
         <v>89</v>
       </c>
       <c r="J176" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="177" spans="1:10">
@@ -8233,9 +8194,6 @@
       <c r="H177" t="s">
         <v>62</v>
       </c>
-      <c r="I177" t="s">
-        <v>679</v>
-      </c>
       <c r="J177" t="s">
         <v>62</v>
       </c>
@@ -8265,9 +8223,6 @@
       <c r="H178" t="s">
         <v>42</v>
       </c>
-      <c r="I178" t="s">
-        <v>679</v>
-      </c>
       <c r="J178" t="s">
         <v>42</v>
       </c>
@@ -8301,7 +8256,7 @@
         <v>89</v>
       </c>
       <c r="J179" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="180" spans="1:10">
@@ -8329,9 +8284,6 @@
       <c r="H180" t="s">
         <v>62</v>
       </c>
-      <c r="I180" t="s">
-        <v>679</v>
-      </c>
       <c r="J180" t="s">
         <v>62</v>
       </c>
@@ -8365,7 +8317,7 @@
         <v>89</v>
       </c>
       <c r="J181" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="182" spans="1:10">
@@ -8397,7 +8349,7 @@
         <v>678</v>
       </c>
       <c r="J182" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="183" spans="1:10">
@@ -8429,7 +8381,7 @@
         <v>678</v>
       </c>
       <c r="J183" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="184" spans="1:10">
@@ -8461,7 +8413,7 @@
         <v>678</v>
       </c>
       <c r="J184" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="185" spans="1:10">
@@ -8493,7 +8445,7 @@
         <v>89</v>
       </c>
       <c r="J185" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="186" spans="1:10">
@@ -8525,7 +8477,7 @@
         <v>678</v>
       </c>
       <c r="J186" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="187" spans="1:10">
@@ -8557,7 +8509,7 @@
         <v>89</v>
       </c>
       <c r="J187" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="188" spans="1:10">
@@ -8589,7 +8541,7 @@
         <v>89</v>
       </c>
       <c r="J188" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="189" spans="1:10">
@@ -8621,7 +8573,7 @@
         <v>89</v>
       </c>
       <c r="J189" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="190" spans="1:10">
@@ -8653,7 +8605,7 @@
         <v>678</v>
       </c>
       <c r="J190" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="191" spans="1:10">
@@ -8685,7 +8637,7 @@
         <v>89</v>
       </c>
       <c r="J191" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="192" spans="1:10">
@@ -8717,7 +8669,7 @@
         <v>678</v>
       </c>
       <c r="J192" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="193" spans="1:10">
@@ -8749,7 +8701,7 @@
         <v>89</v>
       </c>
       <c r="J193" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="194" spans="1:10">
@@ -8777,9 +8729,6 @@
       <c r="H194" t="s">
         <v>644</v>
       </c>
-      <c r="I194" t="s">
-        <v>679</v>
-      </c>
       <c r="J194" t="s">
         <v>644</v>
       </c>
@@ -8813,7 +8762,7 @@
         <v>678</v>
       </c>
       <c r="J195" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="196" spans="1:10">
@@ -8845,7 +8794,7 @@
         <v>89</v>
       </c>
       <c r="J196" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="197" spans="1:10">
@@ -8877,7 +8826,7 @@
         <v>89</v>
       </c>
       <c r="J197" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="198" spans="1:10">
@@ -8909,7 +8858,7 @@
         <v>678</v>
       </c>
       <c r="J198" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
     </row>
     <row r="199" spans="1:10">
@@ -8941,7 +8890,7 @@
         <v>89</v>
       </c>
       <c r="J199" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="200" spans="1:10">
@@ -8973,7 +8922,7 @@
         <v>89</v>
       </c>
       <c r="J200" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="201" spans="1:10">
@@ -9005,7 +8954,7 @@
         <v>89</v>
       </c>
       <c r="J201" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="202" spans="1:10">
@@ -9037,7 +8986,7 @@
         <v>89</v>
       </c>
       <c r="J202" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="203" spans="1:10">
@@ -9069,7 +9018,7 @@
         <v>678</v>
       </c>
       <c r="J203" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="204" spans="1:10">
@@ -9101,7 +9050,7 @@
         <v>678</v>
       </c>
       <c r="J204" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="205" spans="1:10">
@@ -9133,7 +9082,7 @@
         <v>89</v>
       </c>
       <c r="J205" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="206" spans="1:10">
@@ -9165,7 +9114,7 @@
         <v>89</v>
       </c>
       <c r="J206" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="207" spans="1:10">
@@ -9197,7 +9146,7 @@
         <v>678</v>
       </c>
       <c r="J207" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="208" spans="1:10">
@@ -9229,7 +9178,7 @@
         <v>678</v>
       </c>
       <c r="J208" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="209" spans="1:10">
@@ -9261,7 +9210,7 @@
         <v>89</v>
       </c>
       <c r="J209" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="210" spans="1:10">
@@ -9293,7 +9242,7 @@
         <v>678</v>
       </c>
       <c r="J210" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="211" spans="1:10">
@@ -9325,7 +9274,7 @@
         <v>89</v>
       </c>
       <c r="J211" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="212" spans="1:10">
@@ -9357,7 +9306,7 @@
         <v>89</v>
       </c>
       <c r="J212" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="213" spans="1:10">
@@ -9389,7 +9338,7 @@
         <v>89</v>
       </c>
       <c r="J213" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="214" spans="1:10">
@@ -9421,7 +9370,7 @@
         <v>89</v>
       </c>
       <c r="J214" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="215" spans="1:10">
@@ -9449,9 +9398,6 @@
       <c r="H215" t="s">
         <v>42</v>
       </c>
-      <c r="I215" t="s">
-        <v>679</v>
-      </c>
       <c r="J215" t="s">
         <v>42</v>
       </c>
@@ -9485,7 +9431,7 @@
         <v>678</v>
       </c>
       <c r="J216" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="217" spans="1:10">
@@ -9517,7 +9463,7 @@
         <v>678</v>
       </c>
       <c r="J217" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="218" spans="1:10">
@@ -9549,7 +9495,7 @@
         <v>678</v>
       </c>
       <c r="J218" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="219" spans="1:10">
@@ -9581,7 +9527,7 @@
         <v>678</v>
       </c>
       <c r="J219" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="220" spans="1:10">
@@ -9613,7 +9559,7 @@
         <v>89</v>
       </c>
       <c r="J220" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="221" spans="1:10">
@@ -9645,7 +9591,7 @@
         <v>89</v>
       </c>
       <c r="J221" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="222" spans="1:10">
@@ -9677,7 +9623,7 @@
         <v>678</v>
       </c>
       <c r="J222" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="223" spans="1:10">
@@ -9709,7 +9655,7 @@
         <v>89</v>
       </c>
       <c r="J223" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="224" spans="1:10">
@@ -9741,7 +9687,7 @@
         <v>89</v>
       </c>
       <c r="J224" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="225" spans="1:10">
@@ -9773,7 +9719,7 @@
         <v>89</v>
       </c>
       <c r="J225" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="226" spans="1:10">
@@ -9805,7 +9751,7 @@
         <v>678</v>
       </c>
       <c r="J226" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="227" spans="1:10">
@@ -9837,7 +9783,7 @@
         <v>678</v>
       </c>
       <c r="J227" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="228" spans="1:10">
@@ -9869,7 +9815,7 @@
         <v>678</v>
       </c>
       <c r="J228" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
     <row r="229" spans="1:10">
@@ -9897,9 +9843,6 @@
       <c r="H229" t="s">
         <v>644</v>
       </c>
-      <c r="I229" t="s">
-        <v>679</v>
-      </c>
       <c r="J229" t="s">
         <v>644</v>
       </c>
@@ -9933,7 +9876,7 @@
         <v>89</v>
       </c>
       <c r="J230" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="231" spans="1:10">
@@ -9965,7 +9908,7 @@
         <v>89</v>
       </c>
       <c r="J231" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="232" spans="1:10">
@@ -9997,7 +9940,7 @@
         <v>678</v>
       </c>
       <c r="J232" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="233" spans="1:10">
@@ -10029,7 +9972,7 @@
         <v>89</v>
       </c>
       <c r="J233" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="234" spans="1:10">
@@ -10061,7 +10004,7 @@
         <v>89</v>
       </c>
       <c r="J234" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="235" spans="1:10">
@@ -10093,7 +10036,7 @@
         <v>89</v>
       </c>
       <c r="J235" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="236" spans="1:10">
@@ -10125,7 +10068,7 @@
         <v>89</v>
       </c>
       <c r="J236" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="237" spans="1:10">
@@ -10157,7 +10100,7 @@
         <v>89</v>
       </c>
       <c r="J237" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="238" spans="1:10">
@@ -10189,7 +10132,7 @@
         <v>89</v>
       </c>
       <c r="J238" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="239" spans="1:10">
@@ -10221,7 +10164,7 @@
         <v>89</v>
       </c>
       <c r="J239" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="240" spans="1:10">
@@ -10253,7 +10196,7 @@
         <v>89</v>
       </c>
       <c r="J240" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="241" spans="1:10">
@@ -10281,9 +10224,6 @@
       <c r="H241" t="s">
         <v>42</v>
       </c>
-      <c r="I241" t="s">
-        <v>679</v>
-      </c>
       <c r="J241" t="s">
         <v>42</v>
       </c>
@@ -10317,7 +10257,7 @@
         <v>678</v>
       </c>
       <c r="J242" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="243" spans="1:10">
@@ -10349,7 +10289,7 @@
         <v>678</v>
       </c>
       <c r="J243" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="244" spans="1:10">
@@ -10381,7 +10321,7 @@
         <v>89</v>
       </c>
       <c r="J244" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="245" spans="1:10">
@@ -10413,7 +10353,7 @@
         <v>89</v>
       </c>
       <c r="J245" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="246" spans="1:10">
@@ -10445,7 +10385,7 @@
         <v>89</v>
       </c>
       <c r="J246" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="247" spans="1:10">
@@ -10477,7 +10417,7 @@
         <v>89</v>
       </c>
       <c r="J247" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="248" spans="1:10">
@@ -10509,7 +10449,7 @@
         <v>89</v>
       </c>
       <c r="J248" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="249" spans="1:10">
@@ -10541,7 +10481,7 @@
         <v>678</v>
       </c>
       <c r="J249" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="250" spans="1:10">
@@ -10573,7 +10513,7 @@
         <v>678</v>
       </c>
       <c r="J250" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="251" spans="1:10">
@@ -10605,7 +10545,7 @@
         <v>678</v>
       </c>
       <c r="J251" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="252" spans="1:10">
@@ -10637,7 +10577,7 @@
         <v>678</v>
       </c>
       <c r="J252" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="253" spans="1:10">
@@ -10669,7 +10609,7 @@
         <v>89</v>
       </c>
       <c r="J253" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="254" spans="1:10">
@@ -10701,7 +10641,7 @@
         <v>678</v>
       </c>
       <c r="J254" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="255" spans="1:10">
@@ -10733,7 +10673,7 @@
         <v>89</v>
       </c>
       <c r="J255" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="256" spans="1:10">
@@ -10765,7 +10705,7 @@
         <v>678</v>
       </c>
       <c r="J256" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="257" spans="1:10">
@@ -10797,7 +10737,7 @@
         <v>89</v>
       </c>
       <c r="J257" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="258" spans="1:10">
@@ -10829,7 +10769,7 @@
         <v>678</v>
       </c>
       <c r="J258" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="259" spans="1:10">
@@ -10861,7 +10801,7 @@
         <v>678</v>
       </c>
       <c r="J259" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="260" spans="1:10">
@@ -10893,7 +10833,7 @@
         <v>678</v>
       </c>
       <c r="J260" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="261" spans="1:10">
@@ -10925,7 +10865,7 @@
         <v>678</v>
       </c>
       <c r="J261" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="262" spans="1:10">
@@ -10957,7 +10897,7 @@
         <v>89</v>
       </c>
       <c r="J262" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="263" spans="1:10">
@@ -10989,7 +10929,7 @@
         <v>89</v>
       </c>
       <c r="J263" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="264" spans="1:10">
@@ -11021,7 +10961,7 @@
         <v>89</v>
       </c>
       <c r="J264" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="265" spans="1:10">
@@ -11053,7 +10993,7 @@
         <v>678</v>
       </c>
       <c r="J265" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="266" spans="1:10">
@@ -11085,7 +11025,7 @@
         <v>89</v>
       </c>
       <c r="J266" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
     </row>
     <row r="267" spans="1:10">
@@ -11117,7 +11057,7 @@
         <v>89</v>
       </c>
       <c r="J267" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="268" spans="1:10">
@@ -11149,7 +11089,7 @@
         <v>678</v>
       </c>
       <c r="J268" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="269" spans="1:10">
@@ -11181,7 +11121,7 @@
         <v>678</v>
       </c>
       <c r="J269" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="270" spans="1:10">
@@ -11213,7 +11153,7 @@
         <v>89</v>
       </c>
       <c r="J270" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="271" spans="1:10">
@@ -11245,7 +11185,7 @@
         <v>678</v>
       </c>
       <c r="J271" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="272" spans="1:10">
@@ -11277,7 +11217,7 @@
         <v>678</v>
       </c>
       <c r="J272" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="273" spans="1:10">
@@ -11309,7 +11249,7 @@
         <v>89</v>
       </c>
       <c r="J273" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="274" spans="1:10">
@@ -11341,7 +11281,7 @@
         <v>89</v>
       </c>
       <c r="J274" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="275" spans="1:10">
@@ -11373,7 +11313,7 @@
         <v>89</v>
       </c>
       <c r="J275" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="276" spans="1:10">
@@ -11405,7 +11345,7 @@
         <v>89</v>
       </c>
       <c r="J276" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="277" spans="1:10">
@@ -11437,7 +11377,7 @@
         <v>89</v>
       </c>
       <c r="J277" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
     </row>
     <row r="278" spans="1:10">
@@ -11469,7 +11409,7 @@
         <v>89</v>
       </c>
       <c r="J278" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="279" spans="1:10">
@@ -11501,7 +11441,7 @@
         <v>89</v>
       </c>
       <c r="J279" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="280" spans="1:10">
@@ -11533,7 +11473,7 @@
         <v>89</v>
       </c>
       <c r="J280" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="281" spans="1:10">
@@ -11565,7 +11505,7 @@
         <v>89</v>
       </c>
       <c r="J281" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="282" spans="1:10">
@@ -11597,7 +11537,7 @@
         <v>89</v>
       </c>
       <c r="J282" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="283" spans="1:10">
@@ -11629,7 +11569,7 @@
         <v>678</v>
       </c>
       <c r="J283" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="284" spans="1:10">
@@ -11661,7 +11601,7 @@
         <v>89</v>
       </c>
       <c r="J284" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="285" spans="1:10">
@@ -11689,9 +11629,6 @@
       <c r="H285" t="s">
         <v>650</v>
       </c>
-      <c r="I285" t="s">
-        <v>679</v>
-      </c>
       <c r="J285" t="s">
         <v>650</v>
       </c>
@@ -11725,7 +11662,7 @@
         <v>89</v>
       </c>
       <c r="J286" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="287" spans="1:10">
@@ -11757,7 +11694,7 @@
         <v>89</v>
       </c>
       <c r="J287" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
   </sheetData>

</xml_diff>